<commit_message>
proteccion de endpoints lista
</commit_message>
<xml_diff>
--- a/Matriz de Permisos.xlsx
+++ b/Matriz de Permisos.xlsx
@@ -12,14 +12,14 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="4485" windowHeight="7695"/>
   </bookViews>
   <sheets>
-    <sheet name="como quedaria la matriz de perm" sheetId="1" r:id="rId1"/>
+    <sheet name="matriz de permisos" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="29">
   <si>
     <t>Módulo / Recurso</t>
   </si>
@@ -106,19 +106,13 @@
   </si>
   <si>
     <t>Recuperar eliminados (PATCH /restore)</t>
-  </si>
-  <si>
-    <t>Listas</t>
-  </si>
-  <si>
-    <t>Tablas auxiliares / Lookups (GET /listas/*)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -159,8 +153,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -170,18 +171,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -198,35 +187,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -243,6 +232,12 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -261,7 +256,37 @@
         <name val="Arial"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -314,10 +339,10 @@
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="como quedaria la matriz de perm-style" pivot="0" count="4">
-      <tableStyleElement type="wholeTable" size="0" dxfId="6"/>
-      <tableStyleElement type="headerRow" dxfId="5"/>
-      <tableStyleElement type="firstRowStripe" dxfId="4"/>
-      <tableStyleElement type="secondRowStripe" dxfId="3"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="10"/>
+      <tableStyleElement type="headerRow" dxfId="9"/>
+      <tableStyleElement type="firstRowStripe" dxfId="8"/>
+      <tableStyleElement type="secondRowStripe" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -336,13 +361,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Matriz_de_Permisos" displayName="Matriz_de_Permisos" ref="B2:F19" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Matriz_de_Permisos" displayName="Matriz_de_Permisos" ref="B2:F18" headerRowDxfId="6" dataDxfId="0">
   <tableColumns count="5">
-    <tableColumn id="1" name="Módulo / Recurso"/>
-    <tableColumn id="2" name="Acción / Método HTTP"/>
-    <tableColumn id="3" name="Admin"/>
-    <tableColumn id="4" name="Gestor Stock" dataDxfId="1"/>
-    <tableColumn id="5" name="Vendedor" dataDxfId="0"/>
+    <tableColumn id="1" name="Módulo / Recurso" dataDxfId="5"/>
+    <tableColumn id="2" name="Acción / Método HTTP" dataDxfId="4"/>
+    <tableColumn id="3" name="Admin" dataDxfId="3"/>
+    <tableColumn id="4" name="Gestor Stock" dataDxfId="2"/>
+    <tableColumn id="5" name="Vendedor" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="como quedaria la matriz de perm-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -550,331 +575,316 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:I19"/>
+  <dimension ref="B1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.7109375" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="54.85546875" customWidth="1"/>
+    <col min="3" max="3" width="47.28515625" customWidth="1"/>
     <col min="4" max="4" width="14.42578125" customWidth="1"/>
     <col min="5" max="5" width="18.28515625" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" customWidth="1"/>
+    <col min="10" max="11" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="3" t="s">
+    <row r="1" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="8" t="s">
+    <row r="3" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="4"/>
-    </row>
-    <row r="4" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="7" t="s">
+      <c r="D3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="2"/>
+    </row>
+    <row r="4" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="7" t="s">
+      <c r="D4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="6" t="s">
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="6" t="s">
+      <c r="D6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="6" t="s">
+      <c r="D7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="6" t="s">
+      <c r="D8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="7" t="s">
+      <c r="D9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J9" s="6"/>
+    </row>
+    <row r="10" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="7" t="s">
+      <c r="D10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="6" t="s">
+      <c r="D11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
+      <c r="D12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="5" t="s">
+      <c r="D13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="4"/>
-    </row>
-    <row r="15" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
+      <c r="D14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I15" s="4"/>
-    </row>
-    <row r="16" spans="2:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
+      <c r="D15" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="I15" s="2"/>
+    </row>
+    <row r="16" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="D16" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="17" spans="2:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="D17" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="18" spans="2:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="19" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>7</v>
+      <c r="D18" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="E3:F19">
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="E3:F18">
       <formula1>"❌,✅"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
pruebas automatizadas con pytest
</commit_message>
<xml_diff>
--- a/Matriz de Permisos.xlsx
+++ b/Matriz de Permisos.xlsx
@@ -9,17 +9,18 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="4485" windowHeight="7695"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="4485" windowHeight="7695" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="matriz de permisos" sheetId="1" r:id="rId1"/>
+    <sheet name="final " sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="118">
   <si>
     <t>Módulo / Recurso</t>
   </si>
@@ -106,13 +107,280 @@
   </si>
   <si>
     <t>Recuperar eliminados (PATCH /restore)</t>
+  </si>
+  <si>
+    <t>Acción y Ruta</t>
+  </si>
+  <si>
+    <t>Método HTTP</t>
+  </si>
+  <si>
+    <t>Crear almacén (/almacenes/)</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>✔</t>
+  </si>
+  <si>
+    <t>Obtener todos los almacenes (/almacenes/)</t>
+  </si>
+  <si>
+    <t>GET</t>
+  </si>
+  <si>
+    <t>Obtener almacenes activos (/almacenes/activos)</t>
+  </si>
+  <si>
+    <t>Buscar por filtros (/almacenes/filtros)</t>
+  </si>
+  <si>
+    <t>Obtener almacén por ID (/almacenes/{almacen_id})</t>
+  </si>
+  <si>
+    <t>Desactivar almacén (/almacenes/{almacen_id})</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>Activar almacén (/almacenes/activar)</t>
+  </si>
+  <si>
+    <t>PATCH</t>
+  </si>
+  <si>
+    <t>Actualizar almacén (/almacenes/{almacen_id})</t>
+  </si>
+  <si>
+    <t>Asignar producto a almacén (/almacenes/asignar-producto)</t>
+  </si>
+  <si>
+    <t>Ver inventario de almacén (/almacenes/{almacen_id}/inventario)</t>
+  </si>
+  <si>
+    <t>Crear categoría (/categorias/)</t>
+  </si>
+  <si>
+    <t>Obtener todas las categorías (/categorias/)</t>
+  </si>
+  <si>
+    <t>Obtener categorías activas (/categorias/activas)</t>
+  </si>
+  <si>
+    <t>Obtener categoría por ID (/categorias/{categoria_id})</t>
+  </si>
+  <si>
+    <t>Desactivar categoría (/categorias/{categoria_id})</t>
+  </si>
+  <si>
+    <t>Activar categoría (/categorias/{categoria_id}/activar)</t>
+  </si>
+  <si>
+    <t>Editar categoría (/categorias/{categoria_id})</t>
+  </si>
+  <si>
+    <t>Buscar productos por categoría (/categorias/{nombre_categoria}/productos)</t>
+  </si>
+  <si>
+    <t>Obtener todos los clientes (/clientes/)</t>
+  </si>
+  <si>
+    <t>Obtener clientes activos (/clientes/activos)</t>
+  </si>
+  <si>
+    <t>Obtener cliente por ID (/clientes/{id_cliente})</t>
+  </si>
+  <si>
+    <t>Crear cliente (/clientes/)</t>
+  </si>
+  <si>
+    <t>Editar cliente (/clientes/{cliente_id})</t>
+  </si>
+  <si>
+    <t>Desactivar cliente (/clientes/{id_cliente})</t>
+  </si>
+  <si>
+    <t>Activar cliente (/clientes/{id_cliente}/activar)</t>
+  </si>
+  <si>
+    <t>Obtener cliente por cédula (/clientes/cedula/{num_cedula})</t>
+  </si>
+  <si>
+    <t>Obtener ventas de cliente (/clientes/{id_cliente}/ventas)</t>
+  </si>
+  <si>
+    <t>Estadísticas del cliente (/clientes/{id_cliente}/estadisticas)</t>
+  </si>
+  <si>
+    <t>Crear compra (/compras/)</t>
+  </si>
+  <si>
+    <t>Mostrar todas las compras (/compras/)</t>
+  </si>
+  <si>
+    <t>Obtener compra por ID (/compras/{compra_id})</t>
+  </si>
+  <si>
+    <t>Recibir compra (/compras/recibir/{compra_id})</t>
+  </si>
+  <si>
+    <t>Actualizar compra (/compras/{compra_id})</t>
+  </si>
+  <si>
+    <t>Cancelar compra (/compras/{compra_id})</t>
+  </si>
+  <si>
+    <t>Obtener compras por proveedor (/compras/proveedor/{proveedor_id})</t>
+  </si>
+  <si>
+    <t>Reporte de compras por fecha (/compras/reporte/fechas)</t>
+  </si>
+  <si>
+    <t>Crear marca (/marcas/)</t>
+  </si>
+  <si>
+    <t>Obtener todas las marcas (/marcas/)</t>
+  </si>
+  <si>
+    <t>Obtener marcas activas (/marcas/activas)</t>
+  </si>
+  <si>
+    <t>Buscar marca por nombre (/marcas/por/{nombre})</t>
+  </si>
+  <si>
+    <t>Obtener marca por ID (/marcas/{marca_id})</t>
+  </si>
+  <si>
+    <t>Actualizar marca (/marcas/{marca_id})</t>
+  </si>
+  <si>
+    <t>Desactivar marca (/marcas/{marca_id})</t>
+  </si>
+  <si>
+    <t>Activar marca (/marcas/{marca_id}/activar)</t>
+  </si>
+  <si>
+    <t>Estadísticas de la marca (/marcas/{marca_id}/estadisticas)</t>
+  </si>
+  <si>
+    <t>Productos de la marca (/marcas/{marca_id}/productos)</t>
+  </si>
+  <si>
+    <t>Crear producto (/productos/)</t>
+  </si>
+  <si>
+    <t>Obtener todos los productos (/productos/)</t>
+  </si>
+  <si>
+    <t>Obtener productos activos (/productos/activos)</t>
+  </si>
+  <si>
+    <t>Buscar productos por filtros (/productos/filtros)</t>
+  </si>
+  <si>
+    <t>Productos con stock bajo (/productos/stock-bajo)</t>
+  </si>
+  <si>
+    <t>Obtener producto por ID (/productos/{producto_id})</t>
+  </si>
+  <si>
+    <t>Actualizar producto completo (/productos/{producto_id})</t>
+  </si>
+  <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>Editar producto parcial (/productos/{producto_id})</t>
+  </si>
+  <si>
+    <t>Desactivar producto (/productos/{producto_id})</t>
+  </si>
+  <si>
+    <t>Activar producto (/productos/{producto_id}/activar)</t>
+  </si>
+  <si>
+    <t>Asignar producto a almacén (/productos/asignar-almacen)</t>
+  </si>
+  <si>
+    <t>Utilidad del producto (/productos/{producto_id}/utilidad)</t>
+  </si>
+  <si>
+    <t>Crear proveedor (/proveedores/)</t>
+  </si>
+  <si>
+    <t>Obtener proveedores activos (/proveedores/activos)</t>
+  </si>
+  <si>
+    <t>Listar todos los proveedores (/proveedores/)</t>
+  </si>
+  <si>
+    <t>Obtener proveedor por ID (/proveedores/{proveedor_id})</t>
+  </si>
+  <si>
+    <t>Editar proveedor (/proveedores/{proveedor_id})</t>
+  </si>
+  <si>
+    <t>Desactivar proveedor (/proveedores/{proveedor_id})</t>
+  </si>
+  <si>
+    <t>Activar proveedor (/proveedores/activar/{proveedor_id})</t>
+  </si>
+  <si>
+    <t>Buscar proveedores por nombre (/proveedores/filtro/{nombre})</t>
+  </si>
+  <si>
+    <t>Compras por proveedor (/proveedores/{proveedor_id}/compras)</t>
+  </si>
+  <si>
+    <t>Registrar usuario (/usuarios/registrar)</t>
+  </si>
+  <si>
+    <t>Público</t>
+  </si>
+  <si>
+    <t>Inicio de sesión (/usuarios/login)</t>
+  </si>
+  <si>
+    <t>Ver perfil (/usuarios/perfil)</t>
+  </si>
+  <si>
+    <t>Obtener todos los usuarios (/usuarios/)</t>
+  </si>
+  <si>
+    <t>Desactivar usuario (/usuarios/eliminar/{id_user})</t>
+  </si>
+  <si>
+    <t>Crear venta (/ventas/)</t>
+  </si>
+  <si>
+    <t>Listar ventas (/ventas/)</t>
+  </si>
+  <si>
+    <t>Obtener factura por ID (/ventas/ventas/{venta_id})</t>
+  </si>
+  <si>
+    <t>Actualizar venta (/ventas/{venta_id})</t>
+  </si>
+  <si>
+    <t>Ventas por cliente (/ventas/cliente/{cliente_id})</t>
+  </si>
+  <si>
+    <t>Ventas por rango de fechas (/ventas/fecha/)</t>
+  </si>
+  <si>
+    <t>Cancelar venta (/ventas/{venta_id}/cancelar)</t>
+  </si>
+  <si>
+    <t>Reporte diario de ventas (/ventas/reporte/diario)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -160,8 +428,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -171,6 +447,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -187,7 +469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -203,19 +485,14 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -263,6 +540,14 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -361,13 +646,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Matriz_de_Permisos" displayName="Matriz_de_Permisos" ref="B2:F18" headerRowDxfId="6" dataDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Matriz_de_Permisos" displayName="Matriz_de_Permisos" ref="B2:F18" headerRowDxfId="6" dataDxfId="5">
   <tableColumns count="5">
-    <tableColumn id="1" name="Módulo / Recurso" dataDxfId="5"/>
-    <tableColumn id="2" name="Acción / Método HTTP" dataDxfId="4"/>
-    <tableColumn id="3" name="Admin" dataDxfId="3"/>
-    <tableColumn id="4" name="Gestor Stock" dataDxfId="2"/>
-    <tableColumn id="5" name="Vendedor" dataDxfId="1"/>
+    <tableColumn id="1" name="Módulo / Recurso" dataDxfId="4"/>
+    <tableColumn id="2" name="Acción / Método HTTP" dataDxfId="3"/>
+    <tableColumn id="3" name="Admin" dataDxfId="2"/>
+    <tableColumn id="4" name="Gestor Stock" dataDxfId="1"/>
+    <tableColumn id="5" name="Vendedor" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="como quedaria la matriz de perm-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -639,6 +924,7 @@
       <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
+      <c r="H4" s="2"/>
     </row>
     <row r="5" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="5" t="s">
@@ -895,4 +1181,1640 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:G82"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.7109375" customWidth="1"/>
+    <col min="3" max="3" width="66.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B2" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B13" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B14" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B15" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B16" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B17" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B19" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B20" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B22" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B23" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B24" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B25" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B26" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B27" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B28" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B29" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B30" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B31" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G31" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B32" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G32" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="33" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B33" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B34" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B35" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G35" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B36" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B37" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B38" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B39" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B40" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G40" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B41" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G41" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B42" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G42" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B43" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B44" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G44" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B45" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G45" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B46" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G46" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B47" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G47" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="48" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B48" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F48" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G48" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B49" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B50" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G50" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B51" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B52" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E52" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G52" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B53" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G53" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B54" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G54" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B55" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G55" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B56" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G56" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B57" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B58" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B59" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G59" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B60" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G60" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B61" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G61" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B62" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G62" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B63" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F63" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B64" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E64" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F64" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="65" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B65" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G65" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="66" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B66" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E66" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G66" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B67" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F67" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G67" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="68" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B68" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F68" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G68" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="69" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B69" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F69" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G69" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B70" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F70" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G70" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="71" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B71" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="F71" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="G71" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="72" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B72" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E72" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F72" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G72" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="73" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B73" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E73" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G73" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B74" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E74" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F74" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G74" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B75" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E75" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F75" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G75" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B76" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C76" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F76" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G76" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B77" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F77" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G77" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B78" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F78" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B79" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F79" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B80" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E80" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F80" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G80" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B81" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E81" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F81" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G81" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B82" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F82" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G82" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>